<commit_message>
Etapa 1: todos los estribos en Ø3/8 (hechos, proforma Benders) y lista actualizada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Estribos_a_cotizar.xlsx
+++ b/metrados/Estribos_a_cotizar.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t xml:space="preserve">LISTA DE ESTRIBOS A COTIZAR - VIVIENDA UNIFAMILIAR, CHORRILLOS (ETAPA 1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Acero fy 4200. Medidas EXTERIORES del estribo en cm (ancho × alto). Ganchos sísmicos a 135° con extensión ≥ 7.5 cm. Longitud desarrollada incluye ganchos.</t>
+    <t xml:space="preserve">TODOS los estribos en Ø3/8" (cambio de obra). Acero fy 4200. Medidas EXTERIORES en cm (ancho × alto). Ganchos sísmicos a 135° con extensión ≥ 7.5 cm. Longitud incluye ganchos.</t>
   </si>
   <si>
     <t xml:space="preserve">Ítem</t>
@@ -61,7 +61,7 @@
     <t xml:space="preserve">Columnas C-1 y C-2 (10 und)</t>
   </si>
   <si>
-    <t xml:space="preserve">1/2"</t>
+    <t xml:space="preserve">3/8"</t>
   </si>
   <si>
     <t xml:space="preserve">Estribo cerrado rectangular, 2 ganchos 135°</t>
@@ -118,9 +118,6 @@
     <t xml:space="preserve">Vigas de equilibrio VE-1 y VE-2 (16 und)</t>
   </si>
   <si>
-    <t xml:space="preserve">3/8"</t>
-  </si>
-  <si>
     <t xml:space="preserve">22 × 62</t>
   </si>
   <si>
@@ -136,7 +133,7 @@
     <t xml:space="preserve">TOTAL</t>
   </si>
   <si>
-    <t xml:space="preserve">Pendiente: estribos del cerco delantero (plano E-09 aún no recibido). Ø1/2" = ítems 1-6; Ø3/8" = ítems 7-8.</t>
+    <t xml:space="preserve">Pendiente: estribos del cerco (plano E-09 aún no recibido). Ø1/2" ya no se usa en esta lista.</t>
   </si>
   <si>
     <t xml:space="preserve">Cantidad por columna (E-04, piso 1 hasta +2.30): 2×9 en zonas Lo + 13 en empalme @0.075 + 12 resto @0.09 = 43 estribos por columna.</t>
@@ -279,16 +276,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -300,23 +301,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -575,327 +576,327 @@
   <dimension ref="A1:I16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="5" t="n">
         <v>1.48</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="G5" s="5" t="n">
         <v>430</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <f aca="false">ROUNDUP(G5*1.03,0)</f>
         <v>443</v>
       </c>
-      <c r="I5" s="6" t="n">
-        <f aca="false">H5*F5*0.994</f>
-        <v>651.70616</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="I5" s="7" t="n">
+        <f aca="false">H5*F5*0.56</f>
+        <v>367.1584</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.42</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <v>430</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <f aca="false">ROUNDUP(G6*1.03,0)</f>
         <v>443</v>
       </c>
-      <c r="I6" s="6" t="n">
-        <f aca="false">H6*F6*0.994</f>
-        <v>184.94364</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="I6" s="7" t="n">
+        <f aca="false">H6*F6*0.56</f>
+        <v>104.1936</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="5" t="n">
         <v>1.68</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <f aca="false">ROUNDUP(G7*1.03,0)</f>
         <v>89</v>
       </c>
-      <c r="I7" s="6" t="n">
-        <f aca="false">H7*F7*0.994</f>
-        <v>148.62288</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="I7" s="7" t="n">
+        <f aca="false">H7*F7*0.56</f>
+        <v>83.7312</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.99</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="6" t="n">
         <f aca="false">ROUNDUP(G8*1.03,0)</f>
         <v>89</v>
       </c>
-      <c r="I8" s="6" t="n">
-        <f aca="false">H8*F8*0.994</f>
-        <v>87.58134</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="I8" s="7" t="n">
+        <f aca="false">H8*F8*0.56</f>
+        <v>49.3416</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="5" t="n">
         <v>1.78</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <v>129</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="6" t="n">
         <f aca="false">ROUNDUP(G9*1.03,0)</f>
         <v>133</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <f aca="false">H9*F9*0.994</f>
-        <v>235.31956</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="I9" s="7" t="n">
+        <f aca="false">H9*F9*0.56</f>
+        <v>132.5744</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="5" t="n">
         <v>1.26</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="5" t="n">
         <v>129</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="6" t="n">
         <f aca="false">ROUNDUP(G10*1.03,0)</f>
         <v>133</v>
       </c>
-      <c r="I10" s="6" t="n">
-        <f aca="false">H10*F10*0.994</f>
-        <v>166.57452</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="I10" s="7" t="n">
+        <f aca="false">H10*F10*0.56</f>
+        <v>93.8448</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="5" t="n">
         <v>1.93</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <v>381</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="6" t="n">
         <f aca="false">ROUNDUP(G11*1.03,0)</f>
         <v>393</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="I11" s="7" t="n">
         <f aca="false">H11*F11*0.56</f>
         <v>424.7544</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="4" t="n">
+      <c r="F12" s="5" t="n">
         <v>1.18</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="5" t="n">
         <v>86</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="6" t="n">
         <f aca="false">ROUNDUP(G12*1.03,0)</f>
         <v>89</v>
       </c>
-      <c r="I12" s="6" t="n">
+      <c r="I12" s="7" t="n">
         <f aca="false">H12*F12*0.56</f>
         <v>58.8112</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="8" t="n">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="9" t="n">
         <f aca="false">SUM(G5:G12)</f>
         <v>1757</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <f aca="false">SUM(H5:H12)</f>
         <v>1812</v>
       </c>
-      <c r="I13" s="9" t="n">
+      <c r="I13" s="10" t="n">
         <f aca="false">SUM(I5:I12)</f>
-        <v>1958.3137</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+        <v>1314.4096</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>38</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>